<commit_message>
feat(battle): add localized runtime foundation
</commit_message>
<xml_diff>
--- a/DataTables/Datas/__beans__.xlsx
+++ b/DataTables/Datas/__beans__.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace2\luban_examples\MiniTemplate\Datas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52892A95-BBDD-42B6-A9C8-E869A5FA9CB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A78D63-58C4-4421-80A7-C000EDE4DAB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="5535" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
   <si>
     <t>##var</t>
   </si>
@@ -93,6 +93,33 @@
   <si>
     <t>字段变体</t>
     <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>battle.CardEffectBinding</t>
+  </si>
+  <si>
+    <t>:</t>
+  </si>
+  <si>
+    <t>Ordered card effect reference with a semantic text argument.</t>
+  </si>
+  <si>
+    <t>argument_key</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>Named Smart String argument.</t>
+  </si>
+  <si>
+    <t>effect_id</t>
+  </si>
+  <si>
+    <t>int</t>
+  </si>
+  <si>
+    <t>Referenced battle.CardEffect ID.</t>
   </si>
 </sst>
 </file>
@@ -467,7 +494,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="4" width="20.625" customWidth="1"/>
@@ -570,6 +597,41 @@
         <v>22</v>
       </c>
     </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J4" t="s">
+        <v>26</v>
+      </c>
+      <c r="K4" s="2"/>
+      <c r="L4" t="s">
+        <v>27</v>
+      </c>
+      <c r="N4" t="s">
+        <v>28</v>
+      </c>
+      <c r="P4" s="2"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="J5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K5" s="2"/>
+      <c r="L5" t="s">
+        <v>30</v>
+      </c>
+      <c r="N5" t="s">
+        <v>31</v>
+      </c>
+      <c r="P5" s="2"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="J1:P1"/>

</xml_diff>

<commit_message>
feat(battle): integrate UI art and card illustrations
</commit_message>
<xml_diff>
--- a/DataTables/Datas/__beans__.xlsx
+++ b/DataTables/Datas/__beans__.xlsx
@@ -126,7 +126,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -163,8 +163,16 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -180,6 +188,108 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF365F91"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCE6F1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7E6E6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3F7FB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4F8FC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3F9F4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDF9EE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8F4FB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCF5F1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF0F8F8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7F0F8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE6F2E8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7EFCF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEFE7F5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5E9E1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2F1F1"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -204,7 +314,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -216,6 +326,78 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="2" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFill="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="1" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="2" applyAlignment="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -505,132 +687,132 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="5">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="5">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="5">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="5">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="5">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="5">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" t="s" s="5">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" t="s" s="5">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" t="s" s="8">
         <v>10</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" t="s" s="8">
         <v>11</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" t="s" s="8">
         <v>7</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" t="s" s="8">
         <v>6</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O2" t="s" s="8">
         <v>8</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="P2" s="9" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="10">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="10">
         <v>13</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" t="s" s="10">
         <v>14</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" t="s" s="10">
         <v>15</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" t="s" s="10">
         <v>16</v>
       </c>
-      <c r="M3" t="s">
+      <c r="M3" t="s" s="10">
         <v>17</v>
       </c>
-      <c r="N3" t="s">
+      <c r="N3" t="s" s="10">
         <v>18</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="P3" s="11" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B4" t="s">
+      <c r="B4" t="s" s="16">
         <v>23</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" t="s" s="17">
         <v>24</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="18">
         <v>25</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" t="s" s="19">
         <v>26</v>
       </c>
-      <c r="K4" s="2"/>
-      <c r="L4" t="s">
+      <c r="K4" s="20"/>
+      <c r="L4" t="s" s="21">
         <v>27</v>
       </c>
-      <c r="N4" t="s">
+      <c r="N4" t="s" s="16">
         <v>28</v>
       </c>
-      <c r="P4" s="2"/>
+      <c r="P4" s="22"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="J5" t="s">
+      <c r="J5" t="s" s="23">
         <v>29</v>
       </c>
-      <c r="K5" s="2"/>
-      <c r="L5" t="s">
+      <c r="K5" s="24"/>
+      <c r="L5" t="s" s="25">
         <v>30</v>
       </c>
-      <c r="N5" t="s">
+      <c r="N5" t="s" s="26">
         <v>31</v>
       </c>
-      <c r="P5" s="2"/>
+      <c r="P5" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>